<commit_message>
Add tooltips from the ODCS v3.2 schema to all field labels
Every field label in odcs-template.xlsx and odcs-template-v3.2.xlsx now shows
the field's description when selected. Also fixes the Quality Metric tooltip,
which showed the Description text, and typos in the Quality tooltips.
</commit_message>
<xml_diff>
--- a/odcs-template-v3.2.xlsx
+++ b/odcs-template-v3.2.xlsx
@@ -13019,10 +13019,40 @@
       <formula>AND(C$8&lt;&gt;"",IFERROR(INDEX(_ServerFieldMatrix,MATCH($B11,_ServerFieldLabels,0),MATCH(C$8,_ServerTypes,0)),"")="")</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations count="31">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C8:F8" xr:uid="{DA5A2A0C-4ADC-9545-A150-4B9AFA021B81}">
       <formula1>_ServerTypes</formula1>
     </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Server" prompt="Identifier of the server." sqref="A4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Environment" prompt="Environment of the server, e.g., prod, test, dev." sqref="A5"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Description" prompt="Description of the server." sqref="A6"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Type" prompt="Type of the server, e.g., snowflake, databricks, bigquery, postgres, s3, kafka. Selecting a type highlights the required connection details." sqref="A8"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Connection" prompt="Connection details of the server. Which fields are required or optional depends on the server type." sqref="A10"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Account" prompt="Account used by the server, e.g., the Snowflake account." sqref="B11"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Catalog" prompt="Name of the catalog, e.g., the Hive or Unity catalog." sqref="B12"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Catalog URL" prompt="URL of the Iceberg compatible REST catalog service (Polaris, S3 Tables, Nessie, Unity Catalog, Glue, etc.)." sqref="B13"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Database" prompt="Name of the database." sqref="B14"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Dataset" prompt="Name of the dataset, e.g., the GCP dataset name." sqref="B15"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Delimiter" prompt="Only for format = json. How multiple json documents are delimited within one file." sqref="B16"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Encoding" prompt="The expected character encoding for data payloads exposed through this server, for example UTF-8, ISO-8859-1, ASCII or UTF-16." sqref="B17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Endpoint URL" prompt="The server endpoint for S3-compatible servers." sqref="B18"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Format" prompt="File or message format, e.g., parquet, csv, json, delta, avro." sqref="B19"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Host" prompt="Host name or IP address." sqref="B20"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Location" prompt="A URL to a location, e.g., s3://bucket/path/*.parquet. Supports globs where applicable." sqref="B21"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Namespace" prompt="Dot-separated namespace/schema path within the catalog (e.g. db.schema or just db)." sqref="B22"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Path" prompt="Relative or absolute path to the data file(s)." sqref="B23"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Port" prompt="Port to the server. An integer, or a string holding a variable reference such as ${DB_PORT}." sqref="B24"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Project" prompt="Project name, e.g., the GCP project name." sqref="B25"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Region" prompt="Cloud region." sqref="B26"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Region Name" prompt="The region your AWS account uses." sqref="B27"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Schema" prompt="Identify the schema in the data source in which your tables exist." sqref="B28"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Service Name" prompt="Name of the service." sqref="B29"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Staging Directory" prompt="Location in Amazon S3 where Athena stores query results and metadata." sqref="B30"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Stream" prompt="Name of the data stream." sqref="B31"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Warehouse" prompt="Name of the cluster or warehouse, e.g., the Snowflake virtual warehouse." sqref="B32"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Workgroup" prompt="The Athena workgroup to use." sqref="B33"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="ID" prompt="Stable technical identifier for references. Must be unique within its containing array. Cannot contain '.', '#', '/', '\', '@', '!', '%', '&amp;', '^' or whitespace." sqref="B35"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Custom Properties" prompt="A list of key/value pairs for custom properties. Add one row per property: the name in column B, the value in the column of each server." sqref="A37"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -13074,10 +13104,14 @@
       <c r="B7" s="5"/>
     </row>
   </sheetData>
-  <dataValidations disablePrompts="1" count="1">
+  <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" sqref="F4:K6" xr:uid="{7EB39568-B879-514E-B51D-6C44C6D6A95F}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Price Amount" prompt="Subscription price per unit of measure in Price Unit." sqref="A4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Price Currency" prompt="Currency of the subscription price, e.g., USD, EUR." sqref="A5"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Price Unit" prompt="The unit of measure for calculating cost. Examples megabyte, gigabyte." sqref="A6"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Price ID" prompt="Stable technical identifier for references. Must be unique within its containing array. Cannot contain '.', '#', '/', '\', '@', '!', '%', '&amp;', '^' or whitespace." sqref="A7"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -13276,10 +13310,16 @@
       <formula>C5="sql"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations count="7">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A5:A100" xr:uid="{6E57E0C1-DF0C-8D48-991E-BBDF563FC7DE}">
       <formula1>"Contract,Description,Server,Schema,Property,Enum Value,Synonym,Relationship,Quality,Support,Team,Team Member,Role,SLA,Verified Statement,Constraint"</formula1>
     </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Scope" prompt="The element of the contract this definition belongs to, e.g., Contract, Schema, Property, Server, Team." sqref="A4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Scope name" prompt="Name of the element within the scope, e.g., the schema name, or schema.property for a property. Leave empty for Contract." sqref="B4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="URL" prompt="URL to the authority." sqref="C4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Type" prompt="Type of definition for authority: businessDefinition, canonicalUrl, glossary, implementation, ontology, taxonomy, transformationImplementation, tutorial, videoTutorial." sqref="D4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Description" prompt="Description of the authoritative definition for humans." sqref="E4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="ID" prompt="Stable technical identifier for references. Must be unique within its containing array. Cannot contain '.', '#', '/', '\', '@', '!', '%', '&amp;', '^' or whitespace." sqref="F4"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -13538,11 +13578,18 @@
       <formula>C5="sql"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations count="9">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A5:A100" xr:uid="{166C4381-ED4D-5B45-A666-BA1B4BA3B914}">
       <formula1>"contract,schema"</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" sqref="G5:I21" xr:uid="{89C229D8-2F45-3843-936D-0B6A0C8140E9}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Scope" prompt="contract: statement applies to the whole data contract. schema: statement applies to one schema." sqref="A4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Schema name" prompt="Name of the schema, if Scope is schema." sqref="B4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Question" prompt="The canonical question." sqref="C4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Answer" prompt="The expected response or result description. Leave empty for a canonical question without answer." sqref="D4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Tags" prompt="A list of tags to categorize the element, e.g., finance, sensitive, employee_record. Comma-separated." sqref="E4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="ID" prompt="Stable identifier for the entry." sqref="F4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Custom Properties" prompt="A list of key/value pairs for custom properties. Add one column per property: the header is the property name, the cell is the value." sqref="G3"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -13780,11 +13827,17 @@
       <formula>C5="sql"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="2">
+  <dataValidations count="8">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A5:A100" xr:uid="{7B5FEC2C-CDA2-DE49-9323-6490CE349CB2}">
       <formula1>"contract,schema"</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" sqref="F5:H21" xr:uid="{EDCDDD1A-DA2E-B847-956D-CA8A97DFA498}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Scope" prompt="contract: constraint applies to the whole data contract. schema: constraint applies to one schema." sqref="A4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Schema name" prompt="Name of the schema, if Scope is schema." sqref="B4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Constraint" prompt="The constraint text: negative guidance on what AI agents must NOT do with this entity." sqref="C4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Tags" prompt="A list of tags to categorize the element, e.g., finance, sensitive, employee_record. Comma-separated." sqref="D4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="ID" prompt="Stable identifier for the constraint." sqref="E4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Custom Properties" prompt="A list of key/value pairs for custom properties. Add one column per property: the header is the property name, the cell is the value." sqref="F3"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -14064,8 +14117,16 @@
       <formula>C5="sql"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations count="9">
     <dataValidation allowBlank="1" sqref="H5:J21" xr:uid="{95B0536B-A722-0C4C-98F1-D8A0998E5371}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Schema" prompt="Name of the schema containing the property." sqref="A4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Property" prompt="Name of the property whose allowed values are restricted. Use dot notation for nested properties." sqref="B4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Value" prompt="The allowed value. Required." sqref="C4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Label" prompt="Human-readable label for the value, suitable for UI display." sqref="D4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Description" prompt="Optional description of what this enum value represents." sqref="E4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Tags" prompt="A list of tags to categorize the element, e.g., finance, sensitive, employee_record. Comma-separated." sqref="F4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="ID" prompt="Stable technical identifier for references. Must be unique within its containing array. Cannot contain '.', '#', '/', '\', '@', '!', '%', '&amp;', '^' or whitespace." sqref="G4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Custom Properties" prompt="Custom properties attached to this enum value (e.g., translations). Add one column per property: the header is the property name, the cell is the value." sqref="H3"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -14366,8 +14427,17 @@
       <formula>C5="sql"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="1">
+  <dataValidations count="10">
     <dataValidation allowBlank="1" sqref="I5:K21" xr:uid="{8F506C78-426E-8E44-9ADB-6B7B082626E0}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Schema" prompt="Name of the schema." sqref="A4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Property" prompt="Name of the property. Leave empty for a synonym of the schema." sqref="B4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Synonym" prompt="The synonymous term." sqref="C4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Locale" prompt="BCP 47 language tag (e.g., en-US, fr-FR) when the synonym is language-specific." sqref="D4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Source" prompt="Origin of the synonym (e.g., glossary, finance-team, legacy-system)." sqref="E4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Status" prompt="Lifecycle status of the synonym (e.g., active, deprecated)." sqref="F4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Description" prompt="Short human-readable note about when or why this synonym is used." sqref="G4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="ID" prompt="Stable technical identifier for references. Must be unique within its containing array. Cannot contain '.', '#', '/', '\', '@', '!', '%', '&amp;', '^' or whitespace." sqref="H4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Custom Properties" prompt="A list of key/value pairs for custom properties. Add one column per property: the header is the property name, the cell is the value." sqref="I3"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
@@ -14640,7 +14710,7 @@
       <c r="H21" s="5"/>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="11">
     <dataValidation allowBlank="1" sqref="B5:B22 F5:H21 D5:D61" xr:uid="{39D00745-E29F-BB4D-8EFF-9275524C1814}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A5:A100" xr:uid="{9046F39E-9EB3-EF47-83AF-F83388AB159D}">
       <formula1>"Contract,Description,Server,Schema,Property,Enum Value,Synonym,Relationship,Quality,Support,Team,Team Member,Role,SLA,Verified Statement,Constraint"</formula1>
@@ -14648,6 +14718,14 @@
     <dataValidation type="list" allowBlank="1" sqref="E5:E100" xr:uid="{FD2B148B-B740-B14F-B337-F0CE13B025AB}">
       <formula1>"Text,JSON"</formula1>
     </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Scope" prompt="The element of the contract the custom property belongs to, e.g., Contract, Schema, Property, Server, Quality." sqref="A4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Scope Name" prompt="Name of the element within the scope, e.g., the schema name, or schema.property for a property. Leave empty for Contract." sqref="B4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Property" prompt="The name of the key. Names should be in camel case, the same as if they were permanent properties in the contract." sqref="C4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Value" prompt="The value of the key." sqref="D4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Value Type" prompt="Text: the value is kept as a string. JSON: the value is parsed as JSON, e.g., an array or object. Empty: the value is read as YAML would (true is a boolean, 42 a number)." sqref="E4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Description" prompt="Description of the custom property." sqref="F4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Vendor" prompt="Identifies the vendor, provider, or external system associated with this custom property. Lowercase identifier, e.g., confluent, atlan, soda." sqref="G4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="ID" prompt="Stable technical identifier for references. Must be unique within its containing array. Cannot contain '.', '#', '/', '\', '@', '!', '%', '&amp;', '^' or whitespace." sqref="H4"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -15595,7 +15673,7 @@
   <mergeCells count="1">
     <mergeCell ref="A13:B13"/>
   </mergeCells>
-  <dataValidations count="4">
+  <dataValidations count="22">
     <dataValidation type="list" allowBlank="1" sqref="G12:L14 G18:L25" xr:uid="{7EB39568-B879-514E-B51D-6C44C6D6A95F}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
@@ -15604,6 +15682,24 @@
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Owner" prompt="The ID of the team owning the Data Contract._x000a_Required for Data Mesh Manager." sqref="C13" xr:uid="{35986E89-F1AF-D84C-96AD-8E5AC4A64A86}"/>
     <dataValidation allowBlank="1" sqref="C12:C14 C18:C19 C23:C66" xr:uid="{D875F021-2666-244F-B1D7-40151775E3CC}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Kind" prompt="The kind of file this is. Valid value is DataContract." sqref="A4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="apiVersion" prompt="Version of the standard used to build the data contract. Default value is v3.2.0." sqref="A5"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="ID" prompt="A unique identifier used to reduce the risk of dataset name collisions, such as a UUID." sqref="A7"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Name" prompt="Name of the data contract." sqref="A8"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Version" prompt="Current version of the data contract." sqref="A9"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Status" prompt="Current status of the dataset, e.g., proposed, draft, active, deprecated, retired." sqref="A10"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Contract Created" prompt="Timestamp in UTC of when the data contract was created." sqref="A11"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Owner" prompt="The ID of the team owning the data contract." sqref="A13"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Domain" prompt="Name of the logical data domain." sqref="A15"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Data Product" prompt="The name of the data product. DEPRECATED since v3.1.0." sqref="A16"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Tenant" prompt="Indicates the property the data is primarily associated with. Value is case insensitive." sqref="A17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Description" prompt="High level description of the dataset." sqref="A19"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Purpose" prompt="Purpose of the dataset." sqref="B20"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Limitations" prompt="Limitations of the dataset." sqref="B21"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Usage" prompt="Intended usage of the dataset." sqref="B22"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Tags" prompt="A list of tags to categorize the element, e.g., finance, sensitive, employee_record. Comma-separated." sqref="A24"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Context Instructions" prompt="Natural language guidance for AI agents and tools on how to use this entity. Equivalent to a system prompt scoped to this level." sqref="A26"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Context Instructions" prompt="Natural language guidance for AI agents and tools on how to use this entity. Equivalent to a system prompt scoped to this level." sqref="B27"/>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -17900,7 +17996,7 @@
     <mergeCell ref="B11:E11"/>
     <mergeCell ref="B7:E7"/>
   </mergeCells>
-  <dataValidations count="18">
+  <dataValidations count="78">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Unique" prompt="A value must be unique within the dataset" sqref="H18:H53" xr:uid="{274C493E-CBE0-2742-BFD6-A161E5736B5A}">
       <formula1>"true,false"</formula1>
     </dataValidation>
@@ -17945,6 +18041,66 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B7:E7" xr:uid="{235F05D9-F9B3-6C48-A55D-32FE3C7AACA5}">
       <formula1>"object,blob"</formula1>
     </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Name" prompt="Name of the element (e.g., table). Must match the sheet name &quot;Schema &lt;name&gt;&quot;." sqref="A5"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Type" prompt="The physical element data type in the data source, e.g., table, view, topic, file." sqref="A6"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Logical Type" prompt="The logical element data type: object or blob." sqref="A7"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Description" prompt="Description of the element." sqref="A8"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Business Name" prompt="The business name of the element." sqref="A9"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Physical Name" prompt="Physical name of the element in the data source." sqref="A10"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Data Granularity" prompt="Granular level of the data in the object." sqref="A11"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Tags" prompt="A list of tags to categorize the element, e.g., finance, sensitive, employee_record. Comma-separated." sqref="A12"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="ID" prompt="Stable technical identifier for references. Must be unique within its containing array. Cannot contain '.', '#', '/', '\', '@', '!', '%', '&amp;', '^' or whitespace." sqref="A13"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Context (Guidance for AI)" prompt="Natural language guidance for AI agents and tools on how to use this entity. Equivalent to a system prompt scoped to this level." sqref="A14"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Deprecated" prompt="Indicates this element is deprecated and should not be used in new implementations. Defaults to false." sqref="A15"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Logical Type Options" prompt="Additional optional metadata to describe the logical type. Which options apply depends on the logical type." sqref="Y16"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Custom Properties" prompt="A list of key/value pairs for custom properties. Add one column per property: the header is the property name, the cell is the value." sqref="AX16"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Business Name" prompt="The business name of the property." sqref="B17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Logical Type" prompt="The logical element data type: string, number, integer, boolean, array, object, timestamp, date, time, map, or vector." sqref="C17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Physical Type" prompt="The physical element data type in the data source. For example, VARCHAR(2), DOUBLE, INT." sqref="D17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Example(s)" prompt="List of sample element values." sqref="E17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Description" prompt="Description of the property." sqref="F17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Required" prompt="Indicates if the element may contain Null values; possible values are true and false. Default is false." sqref="G17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Unique" prompt="Indicates if the element contains unique values; possible values are true and false. Default is false." sqref="H17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Classification" prompt="Data classification of the element, e.g., confidential, restricted, public, or a more advanced categorization." sqref="I17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Tags" prompt="A list of tags to categorize the element, e.g., finance, sensitive, employee_record. Comma-separated." sqref="J17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Semantic Type" prompt="The semantic role in the data model: column (default) is a physical column; measure is an aggregated value whose expression is in Transform Logic; dimension is a categorical attribute for grouping and filtering." sqref="K17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Deprecated" prompt="Indicates this element is deprecated and should not be used in new implementations. Defaults to false." sqref="L17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Authoritative Definition URL" prompt="URL to a source that provides more details on the element, e.g., a business definition, data catalog, or tutorial." sqref="M17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Authoritative Definition Type" prompt="Type of definition for authority: businessDefinition, canonicalUrl, glossary, implementation, ontology, taxonomy, transformationImplementation, tutorial, videoTutorial." sqref="N17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Physical Name" prompt="Physical name of the property in the data source." sqref="O17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Primary Key" prompt="Boolean value specifying whether the element is primary or not. Default is false." sqref="P17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Primary Key Position" prompt="If element is a primary key, the position of the primary key element. Starts from 1. For account_id, name as primary key, account_id has position 1 and name position 2." sqref="Q17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Partitioned" prompt="Indicates if the element is partitioned; possible values are true and false." sqref="R17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Partition Key Position" prompt="If element is used for partitioning, the position of the partition element. Starts from 1. For country, year as partition columns, country has position 1 and year position 2." sqref="S17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Encrypted Name" prompt="The element name within the dataset that contains the encrypted element value, e.g., email_address_encrypt for email_address." sqref="T17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Transform Sources" prompt="List of objects in the data source used in the transformation." sqref="U17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Transform Logic" prompt="Logic used in the element transformation." sqref="V17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Transform Description" prompt="Describes the transform logic in very simple terms." sqref="W17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Critical Data Element Status" prompt="True or false indicator; if element is considered a critical data element (CDE) then true else false." sqref="X17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Maximum Items" prompt="Maximum number of items (array)." sqref="Y17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Minimum Items" prompt="Minimum number of items (array)." sqref="Z17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Unique Items" prompt="If set to true, all items in the array are unique." sqref="AA17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Format" prompt="string: extra context about the format, e.g., email, uuid. date/timestamp: DateTimeFormatter pattern, e.g., yyyy-MM-dd. integer/number: bit size and sign, following Rust types, e.g., i32, u64, f64." sqref="AB17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Minimum Length" prompt="Minimum length of the string." sqref="AC17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Maximum Length" prompt="Maximum length of the string." sqref="AD17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Exclusive Minimum" prompt="All values must be strictly greater than this value (values &gt; exclusiveMinimum)." sqref="AE17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Minimum" prompt="All values are greater than or equal to this value (values &gt;= minimum)." sqref="AF17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Exclusive Maximum" prompt="All values must be strictly less than this value (values &lt; exclusiveMaximum)." sqref="AG17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Maximum" prompt="All values are less than or equal to this value (values &lt;= maximum)." sqref="AH17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Multiple Of" prompt="Values must be multiples of this number. For example, multiple of 5 has valid values 0, 5, 10, -5." sqref="AI17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Minimum Properties" prompt="Minimum number of properties (object)." sqref="AJ17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Maximum Properties" prompt="Maximum number of properties (object)." sqref="AK17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Required Properties" prompt="Property names that are required to exist in the object." sqref="AL17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Pattern" prompt="Regular expression pattern to define valid values. Follows ECMA-262 regular expression syntax." sqref="AM17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Dimensions" prompt="The fixed length of the vector. Positive integer (only applicable when logical type is vector)." sqref="AN17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Element Type" prompt="Numeric type of each vector element. binary means each element is one bit (binary-quantized vectors)." sqref="AO17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Distance Metric" prompt="Intended similarity metric. Advisory: the physical index may differ." sqref="AP17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Normalized" prompt="True if vectors are L2-normalized before storage, which makes cosine and dotProduct equivalent." sqref="AQ17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Embedding Model" prompt="Identifier of the model used to produce the vectors." sqref="AR17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Embedding Model Version" prompt="Version or revision of the embedding model, when the model identifier does not already carry one." sqref="AS17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Timezone" prompt="Whether the timestamp defines the timezone or not. If true, timezone information is included in the timestamp." sqref="AT17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Default Timezone" prompt="The default timezone of the timestamp. If timezone is not defined, the default timezone UTC is used." sqref="AU17"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="ID" prompt="Stable technical identifier for references. Must be unique within its containing array. Cannot contain '.', '#', '/', '\', '@', '!', '%', '&amp;', '^' or whitespace." sqref="AV17"/>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -18205,10 +18361,9 @@
       <formula>C5="sql"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="8">
+  <dataValidations count="10">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Description" prompt="A human-readable description of the relationship. Explain the business context or purpose of how the source and target are related." sqref="E4" xr:uid="{EE4A1054-F15A-664C-B875-762503081248}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Type" prompt="Type of the relationship column(s)." sqref="B4" xr:uid="{41A27CD9-820D-2E48-B8C9-300C785AF670}"/>
-    <dataValidation allowBlank="1" showErrorMessage="1" sqref="A4 F4" xr:uid="{C01DBA5A-CD2D-5340-88E8-907CC68A70F7}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="From" prompt="Source property or schema of the relationship. Use schema.property dot notation (e.g., orders.customer_id). For composite keys at schema level, use comma-separated values (e.g., orders.order_id, orders.line_id)." sqref="C4" xr:uid="{BF1567BA-BD98-8A43-A618-6A6EA6B0FD4E}"/>
     <dataValidation allowBlank="1" sqref="C22:E42 F5:I21 G22:H40" xr:uid="{8EB79343-A157-4243-B7EE-3C19030C4E99}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Level" prompt="Select if the relationship shall be defined on schema or property level. Use schema level for composite keys." sqref="A5:A100" xr:uid="{64056970-A677-8843-8D33-4CF3120F6E95}">
@@ -18218,6 +18373,9 @@
       <formula1>"foreignKey,references,mapsTo"</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="To" prompt="Target property or schema the source maps to. Use schema.property dot notation (e.g., customers.id). For composite keys at schema level, use comma-separated values matching the order of the 'From' fields." sqref="D4" xr:uid="{7117A4CC-D0A3-894D-B5D8-FA6426CA462E}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Level" prompt="schema: relationship defined at schema level (use for composite keys). property: relationship defined at property level, where From is the current property." sqref="A4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="ID" prompt="Optional stable identifier for this relationship, unique within its containing relationships array. SHOULD remain stable across contract versions." sqref="F4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Custom Properties" prompt="A list of key/value pairs for custom properties. Add one column per property: the header is the property name, the cell is the value." sqref="G3"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -18793,19 +18951,19 @@
       <formula>D5="library"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="16">
+  <dataValidations count="34">
     <dataValidation allowBlank="1" sqref="D22:H42 V5:X21" xr:uid="{E994B14B-32F5-D346-A2D5-4948CC9EA8C3}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Data Quality Type" prompt="Data quality rules support different levels/stages of data quality attributes:_x000a__x000a_Text: A human-readable text that describes the quality of the data._x000a_Library rules: A maintained library of commonly-used predefined quality attributes such as rowCount, unique" sqref="D4" xr:uid="{F5034942-1DBE-6649-8226-7716B942E17B}"/>
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality Scheduler" prompt="Name of the scheduler that runs the quality check, such as cron, Airflow, or Github Action." sqref="M5:N21" xr:uid="{32CE7D0C-23F9-9242-8EB2-22364F11133E}"/>
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality Severity" prompt="The severity of the data quality rule, such as error or warning." sqref="L5:L21" xr:uid="{0F4D661D-23D9-2540-B241-435A8E49610F}"/>
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality Implementation" prompt="The data quality check in the engine's specific format." sqref="K5:K21" xr:uid="{00416CE8-FD1E-374C-B0CF-0FDCB1952802}"/>
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality Engine" prompt="Required for custom DQ rule: name of the third-party engine being used. Any value is authorized here but common values are soda, greatExpectations, montecarlo, etc." sqref="J5:J21" xr:uid="{0459F568-8532-4048-9CA7-5708CD6DF179}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality Threshold Value" prompt="The acutal value for the treshold operator._x000a_For mustBeBetween adn mustNotBeBetween, use [lowerBoundry, upperBoundy] syntax, e.g. [0, 100]." sqref="I5:I21" xr:uid="{E792E24E-6B57-A948-A026-4637119AD944}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Quality Operator" prompt="The comparation operator specifies the condition to validate the rule._x000a_Use it together with the threshold value, e.g. mustBe 0, or mustBeBetween [0,100]_x000a_This is applicable for quality type sql and some library rules." sqref="H5:H21" xr:uid="{15B1EE74-8A6D-3F49-A7EC-55C27203D116}">
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality Threshold Value" prompt="The actual value for the threshold operator._x000a_For mustBeBetween and mustNotBeBetween, use [lowerBoundary, upperBoundary] syntax, e.g. [0, 100]." sqref="I5:I21" xr:uid="{E792E24E-6B57-A948-A026-4637119AD944}"/>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Quality Operator" prompt="The comparison operator specifies the condition to validate the rule._x000a_Use it together with the threshold value, e.g. mustBe 0, or mustBeBetween [0,100]_x000a_This is applicable for quality type sql and some library rules." sqref="H5:H21" xr:uid="{15B1EE74-8A6D-3F49-A7EC-55C27203D116}">
       <formula1>"mustBe, mustNotBe, mustBeGreaterThan, mustBeGreaterOrEqualTo, mustBeLessThan, mustBeLessOrEqualTo, mustBeBetween, mustNotBeBetween"</formula1>
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality Query" prompt="A single SQL query that returns either a numeric or boolean value for comparison. The query must be written in the SQL dialect specific to the provided server. " sqref="G5:G21" xr:uid="{21D55077-EE2C-364C-A32A-00F4CC049BEA}"/>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Quality Metric" prompt="The expected or guaranteed data quality from a business perspective._x000a__x000a_Maps to quality.description" sqref="F5:F21" xr:uid="{FA04105D-EE78-664F-8C72-4098B271EC60}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="Quality Metric" prompt="The predefined data quality metric from the library: nullValues, missingValues, invalidValues, duplicateValues, rowCount._x000a_Only applicable if Quality Type is library or empty." sqref="F5:F21" xr:uid="{FA04105D-EE78-664F-8C72-4098B271EC60}">
       <formula1>"nullValues,missingValues,invalidValues,duplicateValues,rowCount"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="D5:D21" xr:uid="{664F88A2-7556-9B4E-A851-8889D6576B99}">
@@ -18813,11 +18971,29 @@
     </dataValidation>
     <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality" prompt="The expected or guaranteed data quality from a business perspective._x000a__x000a_Maps to quality.description" sqref="E5:E21" xr:uid="{C84C6FF8-FC8D-B848-AC69-3DB82C6CB871}"/>
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Schema" prompt="The schema name must match the name of the schema (table, ...) in the previous sheets." sqref="A4" xr:uid="{67CAE90D-676C-A44B-B965-361A399ACA9A}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Property" prompt="Optional: Leave empty, if this is a schema-level quality check._x000a_The property must match the property name in the schema._x000a_" sqref="B4:C4" xr:uid="{F3E67713-E117-6E46-AEFE-6861F5933838}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Rule" prompt="The predefined data quality rule from the library._x000a_Only appliable if &quot;Quality Type&quot; is set to &quot;library&quot; or empty (which is library by default, if a rule is defined)" sqref="F4" xr:uid="{4E8AA24F-1E70-FF4C-81CC-D9A25B05246C}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Property" prompt="Optional: Leave empty, if this is a schema-level quality check._x000a_The property must match the property name in the schema._x000a_" sqref="B4" xr:uid="{F3E67713-E117-6E46-AEFE-6861F5933838}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Rule" prompt="The predefined data quality rule from the library._x000a_Only applicable if &quot;Quality Type&quot; is set to &quot;library&quot; or empty (which is library by default, if a rule is defined)" sqref="F4" xr:uid="{4E8AA24F-1E70-FF4C-81CC-D9A25B05246C}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P5:P100" xr:uid="{881CD803-6A20-894A-A9FF-DE919EE9E89D}">
       <formula1>"accuracy,completeness,conformity,consistency,coverage,timeliness,uniqueness"</formula1>
     </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Name" prompt="Name of the data quality check." sqref="C4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Description" prompt="Describe the quality check to be completed." sqref="E4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Query (SQL)" prompt="Query string that adheres to the dialect of the provided server. Only applicable if Quality Type is sql." sqref="G4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Threshold Operator" prompt="Comparison operator: mustBe, mustNotBe, mustBeGreaterThan, mustBeGreaterOrEqualTo, mustBeLessThan, mustBeLessOrEqualTo, mustBeBetween, mustNotBeBetween." sqref="H4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Threshold Value" prompt="Value the result is compared to with the threshold operator. For mustBeBetween and mustNotBeBetween, two numbers with the smallest first, e.g., [0, 100]." sqref="I4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Quality Engine (Custom)" prompt="Name of the engine which executes the data quality checks, e.g., soda, greatExpectations. Only applicable if Quality Type is custom." sqref="J4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Implementation (Custom)" prompt="Vendor-specific implementation of the check for the engine. Only applicable if Quality Type is custom." sqref="K4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Severity" prompt="The severity of the quality rule, e.g., info, warning, error." sqref="L4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Scheduler" prompt="The name or type of scheduler used to start the data quality check." sqref="M4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Schedule" prompt="Rule execution schedule details, e.g., a cron expression." sqref="N4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Arguments" prompt="Additional arguments for the metric, if needed, as a JSON object." sqref="O4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Dimension" prompt="The key performance indicator (KPI) or dimension for data quality: accuracy, completeness, conformity, consistency, coverage, timeliness, uniqueness." sqref="P4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Method" prompt="Method used to perform the data quality check." sqref="Q4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Business Impact" prompt="Consequences of the rule failure." sqref="R4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Unit" prompt="Unit the rule is using, popular values are rows or percent, but any value is allowed." sqref="S4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Tags" prompt="A list of tags to categorize the element, e.g., finance, sensitive, employee_record. Comma-separated." sqref="T4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="ID" prompt="Stable technical identifier for references. Must be unique within its containing array. Cannot contain '.', '#', '/', '\', '@', '!', '%', '&amp;', '^' or whitespace." sqref="U4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Custom Properties" prompt="Additional properties required for rule execution. Add one column per property: the header is the property name, the cell is the value." sqref="V3"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -19085,8 +19261,16 @@
       <c r="J21" s="15"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="9">
     <dataValidation allowBlank="1" sqref="B5:F61 G5:J21" xr:uid="{19A11CF7-5A67-E844-8CDE-E9312B26965E}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Channel" prompt="Channel name or identifier." sqref="A4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Channel URL" prompt="Access URL using normal URL scheme (https, mailto, etc.)." sqref="B4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Description" prompt="Description of the channel, free text." sqref="C4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Tool" prompt="Name of the tool: email, slack, teams, discord, ticket, googlechat, or other." sqref="D4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Scope" prompt="Scope can be: interactive, announcements, issues, notifications." sqref="E4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Invitation URL" prompt="Some tools use an invitation URL for requesting or subscribing. Follows the URL scheme." sqref="F4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="ID" prompt="Stable technical identifier for references. Must be unique within its containing array. Cannot contain '.', '#', '/', '\', '@', '!', '%', '&amp;', '^' or whitespace." sqref="G4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Custom Properties" prompt="A list of key/value pairs for custom properties. Add one column per property: the header is the property name, the cell is the value." sqref="H3"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -19423,8 +19607,22 @@
       <c r="L27" s="15"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="15">
     <dataValidation allowBlank="1" sqref="B11:H67 I11:L27" xr:uid="{8BD676B5-0F0C-9D41-BB36-24C33963E434}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Team Name" prompt="Team name." sqref="A4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Description" prompt="Team description." sqref="A5"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Tags" prompt="A list of tags to categorize the element, e.g., finance, sensitive, employee_record. Comma-separated." sqref="A6"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="ID" prompt="Stable technical identifier for references. Must be unique within its containing array. Cannot contain '.', '#', '/', '\', '@', '!', '%', '&amp;', '^' or whitespace." sqref="A7"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Custom Properties" prompt="A list of key/value pairs for custom properties. Add one column per property: the header is the property name, the cell is the value." sqref="J9"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Username" prompt="The user's username or email." sqref="A10"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Name" prompt="The user's name." sqref="B10"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Description" prompt="The user's description." sqref="C10"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Role" prompt="The user's job role; examples might be owner, data steward. There is no limit on the role." sqref="D10"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Tags" prompt="A list of tags to categorize the element, e.g., finance, sensitive, employee_record. Comma-separated." sqref="E10"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Date In" prompt="The date when the user joined the team." sqref="F10"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Date Out" prompt="The date when the user ceased to be part of the team." sqref="G10"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Replaced By Username" prompt="The username of the user who replaced the previous user." sqref="H10"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="ID" prompt="Stable technical identifier for references. Must be unique within its containing array. Cannot contain '.', '#', '/', '\', '@', '!', '%', '&amp;', '^' or whitespace." sqref="I10"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -19715,11 +19913,20 @@
       <c r="K21" s="15"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="11">
     <dataValidation allowBlank="1" sqref="D5:G61 H5:K21" xr:uid="{87F0D0D6-8894-A64F-B36D-300F6FA120B5}"/>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A5:A100" xr:uid="{839C8FC8-93D0-9A4F-BA53-98416339B650}">
       <formula1>"Contract,Server"</formula1>
     </dataValidation>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Scope" prompt="Contract: role applies to the whole data contract. Server: role applies to one server only." sqref="A4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Server name" prompt="Name of the server the role applies to, if Scope is Server." sqref="B4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Role" prompt="Name of the IAM role that provides access to the dataset." sqref="C4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Description" prompt="Description of the IAM role and its permissions." sqref="D4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Access" prompt="The type of access provided by the IAM role, e.g., read, write." sqref="E4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="1st Level Approvers" prompt="The name(s) of the first-level approver(s) of the role." sqref="F4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="2nd Level Approvers" prompt="The name(s) of the second-level approver(s) of the role." sqref="G4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="ID" prompt="Stable technical identifier for references. Must be unique within its containing array. Cannot contain '.', '#', '/', '\', '@', '!', '%', '&amp;', '^' or whitespace." sqref="H4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Custom Properties" prompt="A list of key/value pairs for custom properties. Add one column per property: the header is the property name, the cell is the value." sqref="I3"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -20060,9 +20267,21 @@
       <c r="M23" s="15"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
+  <dataValidations count="14">
     <dataValidation allowBlank="1" sqref="B7:F63 G7:M23" xr:uid="{7F4EE529-7BE7-6547-817C-8DBC88D35FEC}"/>
     <dataValidation allowBlank="1" showErrorMessage="1" sqref="B4" xr:uid="{8220F424-DC29-F648-BD41-E75C77AE8B05}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Default SLA element(s)" prompt="Element (using the element path notation) to do the checks on. DEPRECATED since v3.1, will be removed in ODCS 4.0." sqref="A4"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Custom Properties" prompt="A list of key/value pairs for custom properties. Add one column per property: the header is the property name, the cell is the value." sqref="K5"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Property" prompt="Specific property in SLA, e.g., latency, retention, frequency, availability. May require units." sqref="A6"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Value" prompt="Agreement value. The label will change based on the property itself." sqref="B6"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Extended value" prompt="Extended agreement value. The label will change based on the property itself." sqref="C6"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Unit" prompt="d, day, days for days; y, yr, years for years, etc. Units use the ISO standard." sqref="D6"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Element" prompt="Element(s) to check on. Multiple elements should be extremely rare and, if so, separated by commas." sqref="E6"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Driver" prompt="Describes the importance of the SLA: regulatory, analytics, or operational." sqref="F6"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Description" prompt="Description of the SLA for humans." sqref="G6"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Scheduler" prompt="Name of the scheduler, can be cron or any tool your organization supports." sqref="H6"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="Schedule" prompt="Configuration information for the scheduling tool, for cron a possible value is 0 20 * * *." sqref="I6"/>
+    <dataValidation allowBlank="1" showInputMessage="1" promptTitle="ID" prompt="Stable technical identifier for references. Must be unique within its containing array. Cannot contain '.', '#', '/', '\', '@', '!', '%', '&amp;', '^' or whitespace." sqref="J6"/>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>